<commit_message>
puxando cpf do xlsx
</commit_message>
<xml_diff>
--- a/Test/dados.xlsx
+++ b/Test/dados.xlsx
@@ -13,7 +13,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
-    <t>Nome</t>
+    <t>CPF</t>
   </si>
   <si>
     <t>Idade</t>
@@ -22,7 +22,7 @@
     <t>Curso</t>
   </si>
   <si>
-    <t>Arthur</t>
+    <t>770.396.770-08</t>
   </si>
   <si>
     <t>Dev</t>
@@ -44,7 +44,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -56,13 +56,24 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11.0"/>
+      <color rgb="FFCE9178"/>
+      <name val="Consolas"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F1F1F"/>
+        <bgColor rgb="FF1F1F1F"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -71,11 +82,14 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -294,6 +308,9 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="15.13"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -307,7 +324,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="1">

</xml_diff>

<commit_message>
atualizacao da funcao NovoLancamento
</commit_message>
<xml_diff>
--- a/Test/dados.xlsx
+++ b/Test/dados.xlsx
@@ -11,40 +11,43 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>CPF</t>
-  </si>
-  <si>
-    <t>Idade</t>
-  </si>
-  <si>
-    <t>Curso</t>
-  </si>
-  <si>
-    <t>770.396.770-08</t>
-  </si>
-  <si>
-    <t>Dev</t>
-  </si>
-  <si>
-    <t>Samoel</t>
-  </si>
-  <si>
-    <t>Eng</t>
-  </si>
-  <si>
-    <t>Moreira</t>
-  </si>
-  <si>
-    <t>Mec</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+  <si>
+    <t>Grupo</t>
+  </si>
+  <si>
+    <t>Codigo</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>CNPJ</t>
+  </si>
+  <si>
+    <t>Discriminação</t>
+  </si>
+  <si>
+    <t>08</t>
+  </si>
+  <si>
+    <t>01</t>
+  </si>
+  <si>
+    <t>105 - Brasil</t>
+  </si>
+  <si>
+    <t>0000000</t>
+  </si>
+  <si>
+    <t>BTC - 0,12063421 unidades do criptoativo Bitcoin (BTC) , adquiridas pela corretora BitcoinTrade (28.640.024/0001-24). Custo medio unitario = R$ 137.620,01463737</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -56,24 +59,13 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11.0"/>
-      <color rgb="FFCE9178"/>
-      <name val="Consolas"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1F1F1F"/>
-        <bgColor rgb="FF1F1F1F"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -89,7 +81,7 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -310,6 +302,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="15.13"/>
+    <col customWidth="1" min="5" max="5" width="123.25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -322,38 +315,28 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="1">
-        <v>19.0</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="1">
-        <v>20.0</v>
-      </c>
-      <c r="C3" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="1">
-        <v>21.0</v>
-      </c>
-      <c r="C4" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>8</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fluxo de preenchimento de bens e direitos completo
</commit_message>
<xml_diff>
--- a/Test/dados.xlsx
+++ b/Test/dados.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Grupo</t>
   </si>
@@ -28,6 +28,12 @@
     <t>Discriminação</t>
   </si>
   <si>
+    <t>Sit. 31/12/23</t>
+  </si>
+  <si>
+    <t>Sit. 31/12/24</t>
+  </si>
+  <si>
     <t>08</t>
   </si>
   <si>
@@ -41,6 +47,12 @@
   </si>
   <si>
     <t>BTC - 0,12063421 unidades do criptoativo Bitcoin (BTC) , adquiridas pela corretora BitcoinTrade (28.640.024/0001-24). Custo medio unitario = R$ 137.620,01463737</t>
+  </si>
+  <si>
+    <t>1.200,00</t>
+  </si>
+  <si>
+    <t>1.300,00</t>
   </si>
 </sst>
 </file>
@@ -74,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -83,6 +95,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -302,7 +317,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="15.13"/>
-    <col customWidth="1" min="5" max="5" width="123.25"/>
+    <col customWidth="1" min="5" max="5" width="39.13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -321,22 +336,34 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>